<commit_message>
finish Excel data cleaning!!!!
</commit_message>
<xml_diff>
--- a/Data Cleaning Helper Functions.xlsx
+++ b/Data Cleaning Helper Functions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\torra034\Documents\githubb\NHTSA_Research_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A49CC223-505F-45D9-98F6-6F900BD0DE69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9334B14-EB26-4BAA-A066-AAEA9184F04B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FACB296B-8AC4-4D09-B580-086A78C3F6BA}"/>
   </bookViews>
@@ -2001,6 +2001,7 @@
   <dimension ref="A1:N52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="6" max="6" width="9.140625" customWidth="1"/>
     <col min="7" max="7" width="11.5703125" customWidth="1"/>
     <col min="8" max="8" width="9.140625" customWidth="1"/>
     <col min="9" max="9" width="13.42578125" customWidth="1"/>
@@ -2095,7 +2096,7 @@
         <v>.CSV</v>
       </c>
       <c r="L2" t="str">
-        <f>IF(OR(E2=2007,E2=2008,E2=2022,E2=2023),CONCATENATE(G2,E2,H2,E2,I2,H2,E2,I2,J2,F2,K2),CONCATENATE(G2,E2,H2,E2,I2,J2,F2,K2))</f>
+        <f>IF(OR(E2=2007,E2=2008,E2=2023),CONCATENATE(G2,E2,H2,E2,I2,H2,E2,I2,J2,F2,K2),CONCATENATE(G2,E2,H2,E2,I2,J2,F2,K2))</f>
         <v>Raw Data/2007/FARS2007NationalCSV/FARS2007NationalCSV/ACCIDENT.CSV</v>
       </c>
       <c r="M2" t="str">
@@ -2125,7 +2126,7 @@
         <v>2008</v>
       </c>
       <c r="F3" s="1" t="str">
-        <f t="shared" ref="F3:F52" si="2">IF(E3&lt;=2014,A3,IF(OR(E3=2015,E3=2018,E3=2020,E3=2021,E3=2022,E3=2023),B3,IF(OR(E3=2016,E3=2017),C3,IF(E3=2019,D3,""))))</f>
+        <f>IF(E3&lt;=2014,A3,IF(OR(E3=2015,E3=2018,E3=2020,E3=2021,E3=2022,E3=2023),B3,IF(OR(E3=2016,E3=2017),C3,IF(E3=2019,D3,""))))</f>
         <v>ACCIDENT</v>
       </c>
       <c r="G3" t="s">
@@ -2141,11 +2142,11 @@
         <v>26</v>
       </c>
       <c r="K3" t="str">
-        <f t="shared" ref="K3:K52" si="3">IF(E3&lt;=2021,".CSV",".csv")</f>
+        <f t="shared" ref="K3:K52" si="2">IF(E3&lt;=2021,".CSV",".csv")</f>
         <v>.CSV</v>
       </c>
       <c r="L3" t="str">
-        <f>IF(OR(E3=2007,E3=2008,E3=2022,E3=2023),CONCATENATE(G3,E3,H3,E3,I3,H3,E3,I3,J3,F3,K3),CONCATENATE(G3,E3,H3,E3,I3,J3,F3,K3))</f>
+        <f t="shared" ref="L3:L52" si="3">IF(OR(E3=2007,E3=2008,E3=2023),CONCATENATE(G3,E3,H3,E3,I3,H3,E3,I3,J3,F3,K3),CONCATENATE(G3,E3,H3,E3,I3,J3,F3,K3))</f>
         <v>Raw Data/2008/FARS2008NationalCSV/FARS2008NationalCSV/ACCIDENT.CSV</v>
       </c>
       <c r="M3" t="str">
@@ -2172,7 +2173,7 @@
         <v>2009</v>
       </c>
       <c r="F4" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E4&lt;=2014,A4,IF(OR(E4=2015,E4=2018,E4=2020,E4=2021,E4=2022,E4=2023),B4,IF(OR(E4=2016,E4=2017),C4,IF(E4=2019,D4,""))))</f>
         <v>ACCIDENT</v>
       </c>
       <c r="G4" t="s">
@@ -2188,11 +2189,11 @@
         <v>26</v>
       </c>
       <c r="K4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L4" t="str">
-        <f>IF(OR(E4=2007,E4=2008,E4=2022,E4=2023),CONCATENATE(G4,E4,H4,E4,I4,H4,E4,I4,J4,F4,K4),CONCATENATE(G4,E4,H4,E4,I4,J4,F4,K4))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2009/FARS2009NationalCSV/ACCIDENT.CSV</v>
       </c>
       <c r="M4" t="str">
@@ -2219,7 +2220,7 @@
         <v>2010</v>
       </c>
       <c r="F5" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E5&lt;=2014,A5,IF(OR(E5=2015,E5=2018,E5=2020,E5=2021,E5=2022,E5=2023),B5,IF(OR(E5=2016,E5=2017),C5,IF(E5=2019,D5,""))))</f>
         <v>ACCIDENT</v>
       </c>
       <c r="G5" t="s">
@@ -2235,11 +2236,11 @@
         <v>26</v>
       </c>
       <c r="K5" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L5" t="str">
-        <f>IF(OR(E5=2007,E5=2008,E5=2022,E5=2023),CONCATENATE(G5,E5,H5,E5,I5,H5,E5,I5,J5,F5,K5),CONCATENATE(G5,E5,H5,E5,I5,J5,F5,K5))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2010/FARS2010NationalCSV/ACCIDENT.CSV</v>
       </c>
       <c r="M5" t="str">
@@ -2266,7 +2267,7 @@
         <v>2011</v>
       </c>
       <c r="F6" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E6&lt;=2014,A6,IF(OR(E6=2015,E6=2018,E6=2020,E6=2021,E6=2022,E6=2023),B6,IF(OR(E6=2016,E6=2017),C6,IF(E6=2019,D6,""))))</f>
         <v>ACCIDENT</v>
       </c>
       <c r="G6" t="s">
@@ -2282,11 +2283,11 @@
         <v>26</v>
       </c>
       <c r="K6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L6" t="str">
-        <f>IF(OR(E6=2007,E6=2008,E6=2022,E6=2023),CONCATENATE(G6,E6,H6,E6,I6,H6,E6,I6,J6,F6,K6),CONCATENATE(G6,E6,H6,E6,I6,J6,F6,K6))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2011/FARS2011NationalCSV/ACCIDENT.CSV</v>
       </c>
       <c r="M6" t="str">
@@ -2313,7 +2314,7 @@
         <v>2012</v>
       </c>
       <c r="F7" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E7&lt;=2014,A7,IF(OR(E7=2015,E7=2018,E7=2020,E7=2021,E7=2022,E7=2023),B7,IF(OR(E7=2016,E7=2017),C7,IF(E7=2019,D7,""))))</f>
         <v>ACCIDENT</v>
       </c>
       <c r="G7" t="s">
@@ -2329,11 +2330,11 @@
         <v>26</v>
       </c>
       <c r="K7" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L7" t="str">
-        <f>IF(OR(E7=2007,E7=2008,E7=2022,E7=2023),CONCATENATE(G7,E7,H7,E7,I7,H7,E7,I7,J7,F7,K7),CONCATENATE(G7,E7,H7,E7,I7,J7,F7,K7))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2012/FARS2012NationalCSV/ACCIDENT.CSV</v>
       </c>
       <c r="M7" t="str">
@@ -2360,7 +2361,7 @@
         <v>2013</v>
       </c>
       <c r="F8" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E8&lt;=2014,A8,IF(OR(E8=2015,E8=2018,E8=2020,E8=2021,E8=2022,E8=2023),B8,IF(OR(E8=2016,E8=2017),C8,IF(E8=2019,D8,""))))</f>
         <v>ACCIDENT</v>
       </c>
       <c r="G8" t="s">
@@ -2376,11 +2377,11 @@
         <v>26</v>
       </c>
       <c r="K8" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L8" t="str">
-        <f>IF(OR(E8=2007,E8=2008,E8=2022,E8=2023),CONCATENATE(G8,E8,H8,E8,I8,H8,E8,I8,J8,F8,K8),CONCATENATE(G8,E8,H8,E8,I8,J8,F8,K8))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2013/FARS2013NationalCSV/ACCIDENT.CSV</v>
       </c>
       <c r="M8" t="str">
@@ -2407,7 +2408,7 @@
         <v>2014</v>
       </c>
       <c r="F9" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E9&lt;=2014,A9,IF(OR(E9=2015,E9=2018,E9=2020,E9=2021,E9=2022,E9=2023),B9,IF(OR(E9=2016,E9=2017),C9,IF(E9=2019,D9,""))))</f>
         <v>ACCIDENT</v>
       </c>
       <c r="G9" t="s">
@@ -2423,11 +2424,11 @@
         <v>26</v>
       </c>
       <c r="K9" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L9" t="str">
-        <f>IF(OR(E9=2007,E9=2008,E9=2022,E9=2023),CONCATENATE(G9,E9,H9,E9,I9,H9,E9,I9,J9,F9,K9),CONCATENATE(G9,E9,H9,E9,I9,J9,F9,K9))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2014/FARS2014NationalCSV/ACCIDENT.CSV</v>
       </c>
       <c r="M9" t="str">
@@ -2454,7 +2455,7 @@
         <v>2015</v>
       </c>
       <c r="F10" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E10&lt;=2014,A10,IF(OR(E10=2015,E10=2018,E10=2020,E10=2021,E10=2022,E10=2023),B10,IF(OR(E10=2016,E10=2017),C10,IF(E10=2019,D10,""))))</f>
         <v>accident</v>
       </c>
       <c r="G10" t="s">
@@ -2470,11 +2471,11 @@
         <v>26</v>
       </c>
       <c r="K10" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L10" t="str">
-        <f>IF(OR(E10=2007,E10=2008,E10=2022,E10=2023),CONCATENATE(G10,E10,H10,E10,I10,H10,E10,I10,J10,F10,K10),CONCATENATE(G10,E10,H10,E10,I10,J10,F10,K10))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2015/FARS2015NationalCSV/accident.CSV</v>
       </c>
       <c r="M10" t="str">
@@ -2504,7 +2505,7 @@
         <v>2016</v>
       </c>
       <c r="F11" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E11&lt;=2014,A11,IF(OR(E11=2015,E11=2018,E11=2020,E11=2021,E11=2022,E11=2023),B11,IF(OR(E11=2016,E11=2017),C11,IF(E11=2019,D11,""))))</f>
         <v>accident</v>
       </c>
       <c r="G11" t="s">
@@ -2520,11 +2521,11 @@
         <v>26</v>
       </c>
       <c r="K11" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L11" t="str">
-        <f>IF(OR(E11=2007,E11=2008,E11=2022,E11=2023),CONCATENATE(G11,E11,H11,E11,I11,H11,E11,I11,J11,F11,K11),CONCATENATE(G11,E11,H11,E11,I11,J11,F11,K11))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2016/FARS2016NationalCSV/accident.CSV</v>
       </c>
       <c r="M11" t="str">
@@ -2551,7 +2552,7 @@
         <v>2017</v>
       </c>
       <c r="F12" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E12&lt;=2014,A12,IF(OR(E12=2015,E12=2018,E12=2020,E12=2021,E12=2022,E12=2023),B12,IF(OR(E12=2016,E12=2017),C12,IF(E12=2019,D12,""))))</f>
         <v>accident</v>
       </c>
       <c r="G12" t="s">
@@ -2567,11 +2568,11 @@
         <v>26</v>
       </c>
       <c r="K12" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L12" t="str">
-        <f>IF(OR(E12=2007,E12=2008,E12=2022,E12=2023),CONCATENATE(G12,E12,H12,E12,I12,H12,E12,I12,J12,F12,K12),CONCATENATE(G12,E12,H12,E12,I12,J12,F12,K12))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2017/FARS2017NationalCSV/accident.CSV</v>
       </c>
       <c r="M12" t="str">
@@ -2598,7 +2599,7 @@
         <v>2018</v>
       </c>
       <c r="F13" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E13&lt;=2014,A13,IF(OR(E13=2015,E13=2018,E13=2020,E13=2021,E13=2022,E13=2023),B13,IF(OR(E13=2016,E13=2017),C13,IF(E13=2019,D13,""))))</f>
         <v>accident</v>
       </c>
       <c r="G13" t="s">
@@ -2614,11 +2615,11 @@
         <v>26</v>
       </c>
       <c r="K13" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L13" t="str">
-        <f>IF(OR(E13=2007,E13=2008,E13=2022,E13=2023),CONCATENATE(G13,E13,H13,E13,I13,H13,E13,I13,J13,F13,K13),CONCATENATE(G13,E13,H13,E13,I13,J13,F13,K13))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2018/FARS2018NationalCSV/accident.CSV</v>
       </c>
       <c r="M13" t="str">
@@ -2645,7 +2646,7 @@
         <v>2019</v>
       </c>
       <c r="F14" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E14&lt;=2014,A14,IF(OR(E14=2015,E14=2018,E14=2020,E14=2021,E14=2022,E14=2023),B14,IF(OR(E14=2016,E14=2017),C14,IF(E14=2019,D14,""))))</f>
         <v>accident</v>
       </c>
       <c r="G14" t="s">
@@ -2661,11 +2662,11 @@
         <v>26</v>
       </c>
       <c r="K14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L14" t="str">
-        <f>IF(OR(E14=2007,E14=2008,E14=2022,E14=2023),CONCATENATE(G14,E14,H14,E14,I14,H14,E14,I14,J14,F14,K14),CONCATENATE(G14,E14,H14,E14,I14,J14,F14,K14))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2019/FARS2019NationalCSV/accident.CSV</v>
       </c>
       <c r="M14" t="str">
@@ -2692,7 +2693,7 @@
         <v>2020</v>
       </c>
       <c r="F15" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E15&lt;=2014,A15,IF(OR(E15=2015,E15=2018,E15=2020,E15=2021,E15=2022,E15=2023),B15,IF(OR(E15=2016,E15=2017),C15,IF(E15=2019,D15,""))))</f>
         <v>accident</v>
       </c>
       <c r="G15" t="s">
@@ -2708,11 +2709,11 @@
         <v>26</v>
       </c>
       <c r="K15" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L15" t="str">
-        <f>IF(OR(E15=2007,E15=2008,E15=2022,E15=2023),CONCATENATE(G15,E15,H15,E15,I15,H15,E15,I15,J15,F15,K15),CONCATENATE(G15,E15,H15,E15,I15,J15,F15,K15))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2020/FARS2020NationalCSV/accident.CSV</v>
       </c>
       <c r="M15" t="str">
@@ -2739,7 +2740,7 @@
         <v>2021</v>
       </c>
       <c r="F16" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E16&lt;=2014,A16,IF(OR(E16=2015,E16=2018,E16=2020,E16=2021,E16=2022,E16=2023),B16,IF(OR(E16=2016,E16=2017),C16,IF(E16=2019,D16,""))))</f>
         <v>accident</v>
       </c>
       <c r="G16" t="s">
@@ -2755,11 +2756,11 @@
         <v>26</v>
       </c>
       <c r="K16" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L16" t="str">
-        <f>IF(OR(E16=2007,E16=2008,E16=2022,E16=2023),CONCATENATE(G16,E16,H16,E16,I16,H16,E16,I16,J16,F16,K16),CONCATENATE(G16,E16,H16,E16,I16,J16,F16,K16))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2021/FARS2021NationalCSV/accident.CSV</v>
       </c>
       <c r="M16" t="str">
@@ -2786,7 +2787,7 @@
         <v>2022</v>
       </c>
       <c r="F17" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E17&lt;=2014,A17,IF(OR(E17=2015,E17=2018,E17=2020,E17=2021,E17=2022,E17=2023),B17,IF(OR(E17=2016,E17=2017),C17,IF(E17=2019,D17,""))))</f>
         <v>accident</v>
       </c>
       <c r="G17" t="s">
@@ -2802,16 +2803,16 @@
         <v>26</v>
       </c>
       <c r="K17" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.csv</v>
       </c>
       <c r="L17" t="str">
-        <f>IF(OR(E17=2007,E17=2008,E17=2022,E17=2023),CONCATENATE(G17,E17,H17,E17,I17,H17,E17,I17,J17,F17,K17),CONCATENATE(G17,E17,H17,E17,I17,J17,F17,K17))</f>
-        <v>Raw Data/2022/FARS2022NationalCSV/FARS2022NationalCSV/accident.csv</v>
+        <f t="shared" si="3"/>
+        <v>Raw Data/2022/FARS2022NationalCSV/accident.csv</v>
       </c>
       <c r="M17" t="str">
         <f>CONCATENATE(LOWER(F17),E17," &lt;- ","read.csv(",CHAR(34),L17,CHAR(34),")")</f>
-        <v>accident2022 &lt;- read.csv("Raw Data/2022/FARS2022NationalCSV/FARS2022NationalCSV/accident.csv")</v>
+        <v>accident2022 &lt;- read.csv("Raw Data/2022/FARS2022NationalCSV/accident.csv")</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
@@ -2833,7 +2834,7 @@
         <v>2023</v>
       </c>
       <c r="F18" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E18&lt;=2014,A18,IF(OR(E18=2015,E18=2018,E18=2020,E18=2021,E18=2022,E18=2023),B18,IF(OR(E18=2016,E18=2017),C18,IF(E18=2019,D18,""))))</f>
         <v>accident</v>
       </c>
       <c r="G18" t="s">
@@ -2849,11 +2850,11 @@
         <v>26</v>
       </c>
       <c r="K18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.csv</v>
       </c>
       <c r="L18" t="str">
-        <f>IF(OR(E18=2007,E18=2008,E18=2022,E18=2023),CONCATENATE(G18,E18,H18,E18,I18,H18,E18,I18,J18,F18,K18),CONCATENATE(G18,E18,H18,E18,I18,J18,F18,K18))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2023/FARS2023NationalCSV/FARS2023NationalCSV/accident.csv</v>
       </c>
       <c r="M18" t="str">
@@ -2881,7 +2882,7 @@
         <v>2007</v>
       </c>
       <c r="F19" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E19&lt;=2014,A19,IF(OR(E19=2015,E19=2018,E19=2020,E19=2021,E19=2022,E19=2023),B19,IF(OR(E19=2016,E19=2017),C19,IF(E19=2019,D19,""))))</f>
         <v>PERSON</v>
       </c>
       <c r="G19" t="s">
@@ -2897,11 +2898,11 @@
         <v>26</v>
       </c>
       <c r="K19" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L19" t="str">
-        <f>IF(OR(E19=2007,E19=2008,E19=2022,E19=2023),CONCATENATE(G19,E19,H19,E19,I19,H19,E19,I19,J19,F19,K19),CONCATENATE(G19,E19,H19,E19,I19,J19,F19,K19))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2007/FARS2007NationalCSV/FARS2007NationalCSV/PERSON.CSV</v>
       </c>
       <c r="M19" t="str">
@@ -2929,7 +2930,7 @@
         <v>2008</v>
       </c>
       <c r="F20" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E20&lt;=2014,A20,IF(OR(E20=2015,E20=2018,E20=2020,E20=2021,E20=2022,E20=2023),B20,IF(OR(E20=2016,E20=2017),C20,IF(E20=2019,D20,""))))</f>
         <v>PERSON</v>
       </c>
       <c r="G20" t="s">
@@ -2945,11 +2946,11 @@
         <v>26</v>
       </c>
       <c r="K20" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L20" t="str">
-        <f>IF(OR(E20=2007,E20=2008,E20=2022,E20=2023),CONCATENATE(G20,E20,H20,E20,I20,H20,E20,I20,J20,F20,K20),CONCATENATE(G20,E20,H20,E20,I20,J20,F20,K20))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2008/FARS2008NationalCSV/FARS2008NationalCSV/PERSON.CSV</v>
       </c>
       <c r="M20" t="str">
@@ -2977,7 +2978,7 @@
         <v>2009</v>
       </c>
       <c r="F21" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E21&lt;=2014,A21,IF(OR(E21=2015,E21=2018,E21=2020,E21=2021,E21=2022,E21=2023),B21,IF(OR(E21=2016,E21=2017),C21,IF(E21=2019,D21,""))))</f>
         <v>PERSON</v>
       </c>
       <c r="G21" t="s">
@@ -2993,11 +2994,11 @@
         <v>26</v>
       </c>
       <c r="K21" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L21" t="str">
-        <f>IF(OR(E21=2007,E21=2008,E21=2022,E21=2023),CONCATENATE(G21,E21,H21,E21,I21,H21,E21,I21,J21,F21,K21),CONCATENATE(G21,E21,H21,E21,I21,J21,F21,K21))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2009/FARS2009NationalCSV/PERSON.CSV</v>
       </c>
       <c r="M21" t="str">
@@ -3025,7 +3026,7 @@
         <v>2010</v>
       </c>
       <c r="F22" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E22&lt;=2014,A22,IF(OR(E22=2015,E22=2018,E22=2020,E22=2021,E22=2022,E22=2023),B22,IF(OR(E22=2016,E22=2017),C22,IF(E22=2019,D22,""))))</f>
         <v>PERSON</v>
       </c>
       <c r="G22" t="s">
@@ -3041,11 +3042,11 @@
         <v>26</v>
       </c>
       <c r="K22" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L22" t="str">
-        <f>IF(OR(E22=2007,E22=2008,E22=2022,E22=2023),CONCATENATE(G22,E22,H22,E22,I22,H22,E22,I22,J22,F22,K22),CONCATENATE(G22,E22,H22,E22,I22,J22,F22,K22))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2010/FARS2010NationalCSV/PERSON.CSV</v>
       </c>
       <c r="M22" t="str">
@@ -3073,7 +3074,7 @@
         <v>2011</v>
       </c>
       <c r="F23" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E23&lt;=2014,A23,IF(OR(E23=2015,E23=2018,E23=2020,E23=2021,E23=2022,E23=2023),B23,IF(OR(E23=2016,E23=2017),C23,IF(E23=2019,D23,""))))</f>
         <v>PERSON</v>
       </c>
       <c r="G23" t="s">
@@ -3089,11 +3090,11 @@
         <v>26</v>
       </c>
       <c r="K23" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L23" t="str">
-        <f>IF(OR(E23=2007,E23=2008,E23=2022,E23=2023),CONCATENATE(G23,E23,H23,E23,I23,H23,E23,I23,J23,F23,K23),CONCATENATE(G23,E23,H23,E23,I23,J23,F23,K23))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2011/FARS2011NationalCSV/PERSON.CSV</v>
       </c>
       <c r="M23" t="str">
@@ -3121,7 +3122,7 @@
         <v>2012</v>
       </c>
       <c r="F24" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E24&lt;=2014,A24,IF(OR(E24=2015,E24=2018,E24=2020,E24=2021,E24=2022,E24=2023),B24,IF(OR(E24=2016,E24=2017),C24,IF(E24=2019,D24,""))))</f>
         <v>PERSON</v>
       </c>
       <c r="G24" t="s">
@@ -3137,11 +3138,11 @@
         <v>26</v>
       </c>
       <c r="K24" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L24" t="str">
-        <f>IF(OR(E24=2007,E24=2008,E24=2022,E24=2023),CONCATENATE(G24,E24,H24,E24,I24,H24,E24,I24,J24,F24,K24),CONCATENATE(G24,E24,H24,E24,I24,J24,F24,K24))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2012/FARS2012NationalCSV/PERSON.CSV</v>
       </c>
       <c r="M24" t="str">
@@ -3169,7 +3170,7 @@
         <v>2013</v>
       </c>
       <c r="F25" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E25&lt;=2014,A25,IF(OR(E25=2015,E25=2018,E25=2020,E25=2021,E25=2022,E25=2023),B25,IF(OR(E25=2016,E25=2017),C25,IF(E25=2019,D25,""))))</f>
         <v>PERSON</v>
       </c>
       <c r="G25" t="s">
@@ -3185,11 +3186,11 @@
         <v>26</v>
       </c>
       <c r="K25" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L25" t="str">
-        <f>IF(OR(E25=2007,E25=2008,E25=2022,E25=2023),CONCATENATE(G25,E25,H25,E25,I25,H25,E25,I25,J25,F25,K25),CONCATENATE(G25,E25,H25,E25,I25,J25,F25,K25))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2013/FARS2013NationalCSV/PERSON.CSV</v>
       </c>
       <c r="M25" t="str">
@@ -3217,7 +3218,7 @@
         <v>2014</v>
       </c>
       <c r="F26" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E26&lt;=2014,A26,IF(OR(E26=2015,E26=2018,E26=2020,E26=2021,E26=2022,E26=2023),B26,IF(OR(E26=2016,E26=2017),C26,IF(E26=2019,D26,""))))</f>
         <v>PERSON</v>
       </c>
       <c r="G26" t="s">
@@ -3233,11 +3234,11 @@
         <v>26</v>
       </c>
       <c r="K26" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L26" t="str">
-        <f>IF(OR(E26=2007,E26=2008,E26=2022,E26=2023),CONCATENATE(G26,E26,H26,E26,I26,H26,E26,I26,J26,F26,K26),CONCATENATE(G26,E26,H26,E26,I26,J26,F26,K26))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2014/FARS2014NationalCSV/PERSON.CSV</v>
       </c>
       <c r="M26" t="str">
@@ -3265,7 +3266,7 @@
         <v>2015</v>
       </c>
       <c r="F27" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E27&lt;=2014,A27,IF(OR(E27=2015,E27=2018,E27=2020,E27=2021,E27=2022,E27=2023),B27,IF(OR(E27=2016,E27=2017),C27,IF(E27=2019,D27,""))))</f>
         <v>person</v>
       </c>
       <c r="G27" t="s">
@@ -3281,11 +3282,11 @@
         <v>26</v>
       </c>
       <c r="K27" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L27" t="str">
-        <f>IF(OR(E27=2007,E27=2008,E27=2022,E27=2023),CONCATENATE(G27,E27,H27,E27,I27,H27,E27,I27,J27,F27,K27),CONCATENATE(G27,E27,H27,E27,I27,J27,F27,K27))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2015/FARS2015NationalCSV/person.CSV</v>
       </c>
       <c r="M27" t="str">
@@ -3313,7 +3314,7 @@
         <v>2016</v>
       </c>
       <c r="F28" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E28&lt;=2014,A28,IF(OR(E28=2015,E28=2018,E28=2020,E28=2021,E28=2022,E28=2023),B28,IF(OR(E28=2016,E28=2017),C28,IF(E28=2019,D28,""))))</f>
         <v>Person</v>
       </c>
       <c r="G28" t="s">
@@ -3329,11 +3330,11 @@
         <v>26</v>
       </c>
       <c r="K28" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L28" t="str">
-        <f>IF(OR(E28=2007,E28=2008,E28=2022,E28=2023),CONCATENATE(G28,E28,H28,E28,I28,H28,E28,I28,J28,F28,K28),CONCATENATE(G28,E28,H28,E28,I28,J28,F28,K28))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2016/FARS2016NationalCSV/Person.CSV</v>
       </c>
       <c r="M28" t="str">
@@ -3361,7 +3362,7 @@
         <v>2017</v>
       </c>
       <c r="F29" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E29&lt;=2014,A29,IF(OR(E29=2015,E29=2018,E29=2020,E29=2021,E29=2022,E29=2023),B29,IF(OR(E29=2016,E29=2017),C29,IF(E29=2019,D29,""))))</f>
         <v>Person</v>
       </c>
       <c r="G29" t="s">
@@ -3377,11 +3378,11 @@
         <v>26</v>
       </c>
       <c r="K29" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L29" t="str">
-        <f>IF(OR(E29=2007,E29=2008,E29=2022,E29=2023),CONCATENATE(G29,E29,H29,E29,I29,H29,E29,I29,J29,F29,K29),CONCATENATE(G29,E29,H29,E29,I29,J29,F29,K29))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2017/FARS2017NationalCSV/Person.CSV</v>
       </c>
       <c r="M29" t="str">
@@ -3409,7 +3410,7 @@
         <v>2018</v>
       </c>
       <c r="F30" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E30&lt;=2014,A30,IF(OR(E30=2015,E30=2018,E30=2020,E30=2021,E30=2022,E30=2023),B30,IF(OR(E30=2016,E30=2017),C30,IF(E30=2019,D30,""))))</f>
         <v>person</v>
       </c>
       <c r="G30" t="s">
@@ -3425,11 +3426,11 @@
         <v>26</v>
       </c>
       <c r="K30" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L30" t="str">
-        <f>IF(OR(E30=2007,E30=2008,E30=2022,E30=2023),CONCATENATE(G30,E30,H30,E30,I30,H30,E30,I30,J30,F30,K30),CONCATENATE(G30,E30,H30,E30,I30,J30,F30,K30))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2018/FARS2018NationalCSV/person.CSV</v>
       </c>
       <c r="M30" t="str">
@@ -3457,7 +3458,7 @@
         <v>2019</v>
       </c>
       <c r="F31" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E31&lt;=2014,A31,IF(OR(E31=2015,E31=2018,E31=2020,E31=2021,E31=2022,E31=2023),B31,IF(OR(E31=2016,E31=2017),C31,IF(E31=2019,D31,""))))</f>
         <v>Person</v>
       </c>
       <c r="G31" t="s">
@@ -3473,11 +3474,11 @@
         <v>26</v>
       </c>
       <c r="K31" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L31" t="str">
-        <f>IF(OR(E31=2007,E31=2008,E31=2022,E31=2023),CONCATENATE(G31,E31,H31,E31,I31,H31,E31,I31,J31,F31,K31),CONCATENATE(G31,E31,H31,E31,I31,J31,F31,K31))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2019/FARS2019NationalCSV/Person.CSV</v>
       </c>
       <c r="M31" t="str">
@@ -3505,7 +3506,7 @@
         <v>2020</v>
       </c>
       <c r="F32" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E32&lt;=2014,A32,IF(OR(E32=2015,E32=2018,E32=2020,E32=2021,E32=2022,E32=2023),B32,IF(OR(E32=2016,E32=2017),C32,IF(E32=2019,D32,""))))</f>
         <v>person</v>
       </c>
       <c r="G32" t="s">
@@ -3521,11 +3522,11 @@
         <v>26</v>
       </c>
       <c r="K32" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L32" t="str">
-        <f>IF(OR(E32=2007,E32=2008,E32=2022,E32=2023),CONCATENATE(G32,E32,H32,E32,I32,H32,E32,I32,J32,F32,K32),CONCATENATE(G32,E32,H32,E32,I32,J32,F32,K32))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2020/FARS2020NationalCSV/person.CSV</v>
       </c>
       <c r="M32" t="str">
@@ -3553,7 +3554,7 @@
         <v>2021</v>
       </c>
       <c r="F33" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E33&lt;=2014,A33,IF(OR(E33=2015,E33=2018,E33=2020,E33=2021,E33=2022,E33=2023),B33,IF(OR(E33=2016,E33=2017),C33,IF(E33=2019,D33,""))))</f>
         <v>person</v>
       </c>
       <c r="G33" t="s">
@@ -3569,11 +3570,11 @@
         <v>26</v>
       </c>
       <c r="K33" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L33" t="str">
-        <f>IF(OR(E33=2007,E33=2008,E33=2022,E33=2023),CONCATENATE(G33,E33,H33,E33,I33,H33,E33,I33,J33,F33,K33),CONCATENATE(G33,E33,H33,E33,I33,J33,F33,K33))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2021/FARS2021NationalCSV/person.CSV</v>
       </c>
       <c r="M33" t="str">
@@ -3601,7 +3602,7 @@
         <v>2022</v>
       </c>
       <c r="F34" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E34&lt;=2014,A34,IF(OR(E34=2015,E34=2018,E34=2020,E34=2021,E34=2022,E34=2023),B34,IF(OR(E34=2016,E34=2017),C34,IF(E34=2019,D34,""))))</f>
         <v>person</v>
       </c>
       <c r="G34" t="s">
@@ -3617,16 +3618,16 @@
         <v>26</v>
       </c>
       <c r="K34" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.csv</v>
       </c>
       <c r="L34" t="str">
-        <f>IF(OR(E34=2007,E34=2008,E34=2022,E34=2023),CONCATENATE(G34,E34,H34,E34,I34,H34,E34,I34,J34,F34,K34),CONCATENATE(G34,E34,H34,E34,I34,J34,F34,K34))</f>
-        <v>Raw Data/2022/FARS2022NationalCSV/FARS2022NationalCSV/person.csv</v>
+        <f t="shared" si="3"/>
+        <v>Raw Data/2022/FARS2022NationalCSV/person.csv</v>
       </c>
       <c r="M34" t="str">
         <f>CONCATENATE(LOWER(F34),E34," &lt;- ","read.csv(",CHAR(34),L34,CHAR(34),")")</f>
-        <v>person2022 &lt;- read.csv("Raw Data/2022/FARS2022NationalCSV/FARS2022NationalCSV/person.csv")</v>
+        <v>person2022 &lt;- read.csv("Raw Data/2022/FARS2022NationalCSV/person.csv")</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
@@ -3649,7 +3650,7 @@
         <v>2023</v>
       </c>
       <c r="F35" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E35&lt;=2014,A35,IF(OR(E35=2015,E35=2018,E35=2020,E35=2021,E35=2022,E35=2023),B35,IF(OR(E35=2016,E35=2017),C35,IF(E35=2019,D35,""))))</f>
         <v>person</v>
       </c>
       <c r="G35" t="s">
@@ -3665,11 +3666,11 @@
         <v>26</v>
       </c>
       <c r="K35" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.csv</v>
       </c>
       <c r="L35" t="str">
-        <f>IF(OR(E35=2007,E35=2008,E35=2022,E35=2023),CONCATENATE(G35,E35,H35,E35,I35,H35,E35,I35,J35,F35,K35),CONCATENATE(G35,E35,H35,E35,I35,J35,F35,K35))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2023/FARS2023NationalCSV/FARS2023NationalCSV/person.csv</v>
       </c>
       <c r="M35" t="str">
@@ -3697,7 +3698,7 @@
         <v>2007</v>
       </c>
       <c r="F36" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E36&lt;=2014,A36,IF(OR(E36=2015,E36=2018,E36=2020,E36=2021,E36=2022,E36=2023),B36,IF(OR(E36=2016,E36=2017),C36,IF(E36=2019,D36,""))))</f>
         <v>VEHICLE</v>
       </c>
       <c r="G36" t="s">
@@ -3713,11 +3714,11 @@
         <v>26</v>
       </c>
       <c r="K36" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L36" t="str">
-        <f>IF(OR(E36=2007,E36=2008,E36=2022,E36=2023),CONCATENATE(G36,E36,H36,E36,I36,H36,E36,I36,J36,F36,K36),CONCATENATE(G36,E36,H36,E36,I36,J36,F36,K36))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2007/FARS2007NationalCSV/FARS2007NationalCSV/VEHICLE.CSV</v>
       </c>
       <c r="M36" t="str">
@@ -3745,7 +3746,7 @@
         <v>2008</v>
       </c>
       <c r="F37" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E37&lt;=2014,A37,IF(OR(E37=2015,E37=2018,E37=2020,E37=2021,E37=2022,E37=2023),B37,IF(OR(E37=2016,E37=2017),C37,IF(E37=2019,D37,""))))</f>
         <v>VEHICLE</v>
       </c>
       <c r="G37" t="s">
@@ -3761,11 +3762,11 @@
         <v>26</v>
       </c>
       <c r="K37" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L37" t="str">
-        <f>IF(OR(E37=2007,E37=2008,E37=2022,E37=2023),CONCATENATE(G37,E37,H37,E37,I37,H37,E37,I37,J37,F37,K37),CONCATENATE(G37,E37,H37,E37,I37,J37,F37,K37))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2008/FARS2008NationalCSV/FARS2008NationalCSV/VEHICLE.CSV</v>
       </c>
       <c r="M37" t="str">
@@ -3793,7 +3794,7 @@
         <v>2009</v>
       </c>
       <c r="F38" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E38&lt;=2014,A38,IF(OR(E38=2015,E38=2018,E38=2020,E38=2021,E38=2022,E38=2023),B38,IF(OR(E38=2016,E38=2017),C38,IF(E38=2019,D38,""))))</f>
         <v>VEHICLE</v>
       </c>
       <c r="G38" t="s">
@@ -3809,11 +3810,11 @@
         <v>26</v>
       </c>
       <c r="K38" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L38" t="str">
-        <f>IF(OR(E38=2007,E38=2008,E38=2022,E38=2023),CONCATENATE(G38,E38,H38,E38,I38,H38,E38,I38,J38,F38,K38),CONCATENATE(G38,E38,H38,E38,I38,J38,F38,K38))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2009/FARS2009NationalCSV/VEHICLE.CSV</v>
       </c>
       <c r="M38" t="str">
@@ -3841,7 +3842,7 @@
         <v>2010</v>
       </c>
       <c r="F39" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E39&lt;=2014,A39,IF(OR(E39=2015,E39=2018,E39=2020,E39=2021,E39=2022,E39=2023),B39,IF(OR(E39=2016,E39=2017),C39,IF(E39=2019,D39,""))))</f>
         <v>VEHICLE</v>
       </c>
       <c r="G39" t="s">
@@ -3857,11 +3858,11 @@
         <v>26</v>
       </c>
       <c r="K39" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L39" t="str">
-        <f>IF(OR(E39=2007,E39=2008,E39=2022,E39=2023),CONCATENATE(G39,E39,H39,E39,I39,H39,E39,I39,J39,F39,K39),CONCATENATE(G39,E39,H39,E39,I39,J39,F39,K39))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2010/FARS2010NationalCSV/VEHICLE.CSV</v>
       </c>
       <c r="M39" t="str">
@@ -3889,7 +3890,7 @@
         <v>2011</v>
       </c>
       <c r="F40" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E40&lt;=2014,A40,IF(OR(E40=2015,E40=2018,E40=2020,E40=2021,E40=2022,E40=2023),B40,IF(OR(E40=2016,E40=2017),C40,IF(E40=2019,D40,""))))</f>
         <v>VEHICLE</v>
       </c>
       <c r="G40" t="s">
@@ -3905,11 +3906,11 @@
         <v>26</v>
       </c>
       <c r="K40" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L40" t="str">
-        <f>IF(OR(E40=2007,E40=2008,E40=2022,E40=2023),CONCATENATE(G40,E40,H40,E40,I40,H40,E40,I40,J40,F40,K40),CONCATENATE(G40,E40,H40,E40,I40,J40,F40,K40))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2011/FARS2011NationalCSV/VEHICLE.CSV</v>
       </c>
       <c r="M40" t="str">
@@ -3937,7 +3938,7 @@
         <v>2012</v>
       </c>
       <c r="F41" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E41&lt;=2014,A41,IF(OR(E41=2015,E41=2018,E41=2020,E41=2021,E41=2022,E41=2023),B41,IF(OR(E41=2016,E41=2017),C41,IF(E41=2019,D41,""))))</f>
         <v>VEHICLE</v>
       </c>
       <c r="G41" t="s">
@@ -3953,11 +3954,11 @@
         <v>26</v>
       </c>
       <c r="K41" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L41" t="str">
-        <f>IF(OR(E41=2007,E41=2008,E41=2022,E41=2023),CONCATENATE(G41,E41,H41,E41,I41,H41,E41,I41,J41,F41,K41),CONCATENATE(G41,E41,H41,E41,I41,J41,F41,K41))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2012/FARS2012NationalCSV/VEHICLE.CSV</v>
       </c>
       <c r="M41" t="str">
@@ -3985,7 +3986,7 @@
         <v>2013</v>
       </c>
       <c r="F42" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E42&lt;=2014,A42,IF(OR(E42=2015,E42=2018,E42=2020,E42=2021,E42=2022,E42=2023),B42,IF(OR(E42=2016,E42=2017),C42,IF(E42=2019,D42,""))))</f>
         <v>VEHICLE</v>
       </c>
       <c r="G42" t="s">
@@ -4001,11 +4002,11 @@
         <v>26</v>
       </c>
       <c r="K42" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L42" t="str">
-        <f>IF(OR(E42=2007,E42=2008,E42=2022,E42=2023),CONCATENATE(G42,E42,H42,E42,I42,H42,E42,I42,J42,F42,K42),CONCATENATE(G42,E42,H42,E42,I42,J42,F42,K42))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2013/FARS2013NationalCSV/VEHICLE.CSV</v>
       </c>
       <c r="M42" t="str">
@@ -4033,7 +4034,7 @@
         <v>2014</v>
       </c>
       <c r="F43" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E43&lt;=2014,A43,IF(OR(E43=2015,E43=2018,E43=2020,E43=2021,E43=2022,E43=2023),B43,IF(OR(E43=2016,E43=2017),C43,IF(E43=2019,D43,""))))</f>
         <v>VEHICLE</v>
       </c>
       <c r="G43" t="s">
@@ -4049,11 +4050,11 @@
         <v>26</v>
       </c>
       <c r="K43" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L43" t="str">
-        <f>IF(OR(E43=2007,E43=2008,E43=2022,E43=2023),CONCATENATE(G43,E43,H43,E43,I43,H43,E43,I43,J43,F43,K43),CONCATENATE(G43,E43,H43,E43,I43,J43,F43,K43))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2014/FARS2014NationalCSV/VEHICLE.CSV</v>
       </c>
       <c r="M43" t="str">
@@ -4081,7 +4082,7 @@
         <v>2015</v>
       </c>
       <c r="F44" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E44&lt;=2014,A44,IF(OR(E44=2015,E44=2018,E44=2020,E44=2021,E44=2022,E44=2023),B44,IF(OR(E44=2016,E44=2017),C44,IF(E44=2019,D44,""))))</f>
         <v>vehicle</v>
       </c>
       <c r="G44" t="s">
@@ -4097,11 +4098,11 @@
         <v>26</v>
       </c>
       <c r="K44" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L44" t="str">
-        <f>IF(OR(E44=2007,E44=2008,E44=2022,E44=2023),CONCATENATE(G44,E44,H44,E44,I44,H44,E44,I44,J44,F44,K44),CONCATENATE(G44,E44,H44,E44,I44,J44,F44,K44))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2015/FARS2015NationalCSV/vehicle.CSV</v>
       </c>
       <c r="M44" t="str">
@@ -4129,7 +4130,7 @@
         <v>2016</v>
       </c>
       <c r="F45" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E45&lt;=2014,A45,IF(OR(E45=2015,E45=2018,E45=2020,E45=2021,E45=2022,E45=2023),B45,IF(OR(E45=2016,E45=2017),C45,IF(E45=2019,D45,""))))</f>
         <v>Vehicle</v>
       </c>
       <c r="G45" t="s">
@@ -4145,11 +4146,11 @@
         <v>26</v>
       </c>
       <c r="K45" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L45" t="str">
-        <f>IF(OR(E45=2007,E45=2008,E45=2022,E45=2023),CONCATENATE(G45,E45,H45,E45,I45,H45,E45,I45,J45,F45,K45),CONCATENATE(G45,E45,H45,E45,I45,J45,F45,K45))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2016/FARS2016NationalCSV/Vehicle.CSV</v>
       </c>
       <c r="M45" t="str">
@@ -4177,7 +4178,7 @@
         <v>2017</v>
       </c>
       <c r="F46" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E46&lt;=2014,A46,IF(OR(E46=2015,E46=2018,E46=2020,E46=2021,E46=2022,E46=2023),B46,IF(OR(E46=2016,E46=2017),C46,IF(E46=2019,D46,""))))</f>
         <v>Vehicle</v>
       </c>
       <c r="G46" t="s">
@@ -4193,11 +4194,11 @@
         <v>26</v>
       </c>
       <c r="K46" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L46" t="str">
-        <f>IF(OR(E46=2007,E46=2008,E46=2022,E46=2023),CONCATENATE(G46,E46,H46,E46,I46,H46,E46,I46,J46,F46,K46),CONCATENATE(G46,E46,H46,E46,I46,J46,F46,K46))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2017/FARS2017NationalCSV/Vehicle.CSV</v>
       </c>
       <c r="M46" t="str">
@@ -4225,7 +4226,7 @@
         <v>2018</v>
       </c>
       <c r="F47" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E47&lt;=2014,A47,IF(OR(E47=2015,E47=2018,E47=2020,E47=2021,E47=2022,E47=2023),B47,IF(OR(E47=2016,E47=2017),C47,IF(E47=2019,D47,""))))</f>
         <v>vehicle</v>
       </c>
       <c r="G47" t="s">
@@ -4241,11 +4242,11 @@
         <v>26</v>
       </c>
       <c r="K47" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L47" t="str">
-        <f>IF(OR(E47=2007,E47=2008,E47=2022,E47=2023),CONCATENATE(G47,E47,H47,E47,I47,H47,E47,I47,J47,F47,K47),CONCATENATE(G47,E47,H47,E47,I47,J47,F47,K47))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2018/FARS2018NationalCSV/vehicle.CSV</v>
       </c>
       <c r="M47" t="str">
@@ -4273,7 +4274,7 @@
         <v>2019</v>
       </c>
       <c r="F48" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E48&lt;=2014,A48,IF(OR(E48=2015,E48=2018,E48=2020,E48=2021,E48=2022,E48=2023),B48,IF(OR(E48=2016,E48=2017),C48,IF(E48=2019,D48,""))))</f>
         <v>vehicle</v>
       </c>
       <c r="G48" t="s">
@@ -4289,11 +4290,11 @@
         <v>26</v>
       </c>
       <c r="K48" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L48" t="str">
-        <f>IF(OR(E48=2007,E48=2008,E48=2022,E48=2023),CONCATENATE(G48,E48,H48,E48,I48,H48,E48,I48,J48,F48,K48),CONCATENATE(G48,E48,H48,E48,I48,J48,F48,K48))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2019/FARS2019NationalCSV/vehicle.CSV</v>
       </c>
       <c r="M48" t="str">
@@ -4321,7 +4322,7 @@
         <v>2020</v>
       </c>
       <c r="F49" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E49&lt;=2014,A49,IF(OR(E49=2015,E49=2018,E49=2020,E49=2021,E49=2022,E49=2023),B49,IF(OR(E49=2016,E49=2017),C49,IF(E49=2019,D49,""))))</f>
         <v>vehicle</v>
       </c>
       <c r="G49" t="s">
@@ -4337,11 +4338,11 @@
         <v>26</v>
       </c>
       <c r="K49" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L49" t="str">
-        <f>IF(OR(E49=2007,E49=2008,E49=2022,E49=2023),CONCATENATE(G49,E49,H49,E49,I49,H49,E49,I49,J49,F49,K49),CONCATENATE(G49,E49,H49,E49,I49,J49,F49,K49))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2020/FARS2020NationalCSV/vehicle.CSV</v>
       </c>
       <c r="M49" t="str">
@@ -4369,7 +4370,7 @@
         <v>2021</v>
       </c>
       <c r="F50" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E50&lt;=2014,A50,IF(OR(E50=2015,E50=2018,E50=2020,E50=2021,E50=2022,E50=2023),B50,IF(OR(E50=2016,E50=2017),C50,IF(E50=2019,D50,""))))</f>
         <v>vehicle</v>
       </c>
       <c r="G50" t="s">
@@ -4385,11 +4386,11 @@
         <v>26</v>
       </c>
       <c r="K50" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.CSV</v>
       </c>
       <c r="L50" t="str">
-        <f>IF(OR(E50=2007,E50=2008,E50=2022,E50=2023),CONCATENATE(G50,E50,H50,E50,I50,H50,E50,I50,J50,F50,K50),CONCATENATE(G50,E50,H50,E50,I50,J50,F50,K50))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2021/FARS2021NationalCSV/vehicle.CSV</v>
       </c>
       <c r="M50" t="str">
@@ -4417,7 +4418,7 @@
         <v>2022</v>
       </c>
       <c r="F51" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E51&lt;=2014,A51,IF(OR(E51=2015,E51=2018,E51=2020,E51=2021,E51=2022,E51=2023),B51,IF(OR(E51=2016,E51=2017),C51,IF(E51=2019,D51,""))))</f>
         <v>vehicle</v>
       </c>
       <c r="G51" t="s">
@@ -4433,16 +4434,16 @@
         <v>26</v>
       </c>
       <c r="K51" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.csv</v>
       </c>
       <c r="L51" t="str">
-        <f>IF(OR(E51=2007,E51=2008,E51=2022,E51=2023),CONCATENATE(G51,E51,H51,E51,I51,H51,E51,I51,J51,F51,K51),CONCATENATE(G51,E51,H51,E51,I51,J51,F51,K51))</f>
-        <v>Raw Data/2022/FARS2022NationalCSV/FARS2022NationalCSV/vehicle.csv</v>
+        <f t="shared" si="3"/>
+        <v>Raw Data/2022/FARS2022NationalCSV/vehicle.csv</v>
       </c>
       <c r="M51" t="str">
         <f>CONCATENATE(LOWER(F51),E51," &lt;- ","read.csv(",CHAR(34),L51,CHAR(34),")")</f>
-        <v>vehicle2022 &lt;- read.csv("Raw Data/2022/FARS2022NationalCSV/FARS2022NationalCSV/vehicle.csv")</v>
+        <v>vehicle2022 &lt;- read.csv("Raw Data/2022/FARS2022NationalCSV/vehicle.csv")</v>
       </c>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.25">
@@ -4465,7 +4466,7 @@
         <v>2023</v>
       </c>
       <c r="F52" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(E52&lt;=2014,A52,IF(OR(E52=2015,E52=2018,E52=2020,E52=2021,E52=2022,E52=2023),B52,IF(OR(E52=2016,E52=2017),C52,IF(E52=2019,D52,""))))</f>
         <v>vehicle</v>
       </c>
       <c r="G52" t="s">
@@ -4481,11 +4482,11 @@
         <v>26</v>
       </c>
       <c r="K52" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>.csv</v>
       </c>
       <c r="L52" t="str">
-        <f>IF(OR(E52=2007,E52=2008,E52=2022,E52=2023),CONCATENATE(G52,E52,H52,E52,I52,H52,E52,I52,J52,F52,K52),CONCATENATE(G52,E52,H52,E52,I52,J52,F52,K52))</f>
+        <f t="shared" si="3"/>
         <v>Raw Data/2023/FARS2023NationalCSV/FARS2023NationalCSV/vehicle.csv</v>
       </c>
       <c r="M52" t="str">

</xml_diff>